<commit_message>
rerun everything after the review
</commit_message>
<xml_diff>
--- a/01_Trunk/03_Quantification/c_data/quantification.xlsx
+++ b/01_Trunk/03_Quantification/c_data/quantification.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4444" uniqueCount="4047">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4441" uniqueCount="4045">
   <si>
     <t>sheet</t>
   </si>
@@ -12156,12 +12156,6 @@
   </si>
   <si>
     <t>3.0.2</t>
-  </si>
-  <si>
-    <t>writexl</t>
-  </si>
-  <si>
-    <t>2.0.1</t>
   </si>
 </sst>
 </file>
@@ -67307,7 +67301,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -67926,17 +67920,6 @@
         <v>3939</v>
       </c>
     </row>
-    <row r="57" spans="1:3">
-      <c r="A57" t="s">
-        <v>4045</v>
-      </c>
-      <c r="B57" t="s">
-        <v>4046</v>
-      </c>
-      <c r="C57" t="s">
-        <v>4019</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>